<commit_message>
paper run 2026-09-05 11:54
</commit_message>
<xml_diff>
--- a/reports/2026-09-05.xlsx
+++ b/reports/2026-09-05.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,49 @@
       </c>
       <c r="K2" t="n">
         <v>-38.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:12:54.310877+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.789</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.00103</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>-2.94</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +593,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -570,7 +613,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -590,7 +633,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-38.8</v>
+        <v>-41.74</v>
       </c>
     </row>
     <row r="7">
@@ -610,7 +653,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-38.8</v>
+        <v>-41.74</v>
       </c>
     </row>
     <row r="9">
@@ -630,7 +673,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>737.2200000000001</v>
+        <v>734.2800000000001</v>
       </c>
     </row>
     <row r="12">
@@ -677,149 +720,168 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>-38.8</v>
+        <v>-11.24</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>-2.94</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-38.8</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
-        <v>-38.8</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-50.04</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-2.94</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>-38.8</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-75.66</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-2.94</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>-38.8</v>
+        <v>25.62</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>25.62</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-75.66</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-2.94</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" t="n">
-        <v>-38.8</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>По окнам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -841,23 +903,23 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>-38.8</v>
+        <v>-41.74</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -879,7 +941,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -889,121 +951,207 @@
         <v>0</v>
       </c>
       <c r="D32" t="n">
+        <v>-2.94</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
         <v>-38.8</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" t="n">
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
         <v>-38.8</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>-2.94</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" t="n">
-        <v>-38.8</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-41.74</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>-41.74</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" t="n">
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
         <v>-38.8</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-2.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-05 17:53
</commit_message>
<xml_diff>
--- a/reports/2026-09-05.xlsx
+++ b/reports/2026-09-05.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,49 @@
       </c>
       <c r="K3" t="n">
         <v>-2.94</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-05T17:23:56.682655+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F4" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>40</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.00111</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>19.6</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +636,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -623,7 +666,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="6">
@@ -633,7 +676,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-41.74</v>
+        <v>-22.14</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +686,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="8">
@@ -663,7 +706,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="10">
@@ -673,7 +716,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>734.2800000000001</v>
+        <v>753.8800000000001</v>
       </c>
     </row>
     <row r="12">
@@ -724,13 +767,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>-11.24</v>
+        <v>-47.95</v>
       </c>
       <c r="E15" t="n">
         <v>-2.94</v>
@@ -743,16 +786,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>-38.8</v>
+        <v>-3.52</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="17">
@@ -765,307 +808,320 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>-50.04</v>
+        <v>-1.43</v>
       </c>
       <c r="E18" t="n">
-        <v>-2.94</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-50.04</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-2.94</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
-        <v>-75.66</v>
-      </c>
-      <c r="E20" t="n">
-        <v>-2.94</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
         <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>25.62</v>
+        <v>-77.09</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>16.66</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>25.62</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" t="n">
-        <v>25.62</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NO_LIQUIDITY</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>2</v>
       </c>
       <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-11.09</v>
+      </c>
+      <c r="E24" t="n">
         <v>0</v>
       </c>
-      <c r="D24" t="n">
-        <v>-75.66</v>
-      </c>
-      <c r="E24" t="n">
-        <v>-2.94</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-40.38</v>
+      </c>
+      <c r="E25" t="n">
+        <v>16.66</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>2</v>
-      </c>
-      <c r="C29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" t="n">
-        <v>-41.74</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>19.6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="n">
         <v>0</v>
       </c>
-      <c r="D32" t="n">
-        <v>-2.94</v>
+      <c r="D31" t="n">
+        <v>-41.74</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5m</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
         <v>0</v>
       </c>
-      <c r="D33" t="n">
-        <v>-38.8</v>
+      <c r="D34" t="n">
+        <v>-2.94</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" t="n">
-        <v>-38.8</v>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-19.2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
         <v>0</v>
       </c>
-      <c r="D37" t="n">
-        <v>-2.94</v>
+      <c r="D38" t="n">
+        <v>-38.8</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>-2.94</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>-41.74</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>По силе движения</t>
+          <t>По цене входа</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1087,23 +1143,23 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>-41.74</v>
+        <v>-22.14</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>По направлению</t>
+          <t>По силе движения</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1125,33 +1181,71 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-22.14</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" t="n">
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
         <v>0</v>
       </c>
-      <c r="D46" t="n">
+      <c r="D49" t="n">
         <v>-38.8</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B47" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" t="n">
-        <v>-2.94</v>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>16.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-05 23:52
</commit_message>
<xml_diff>
--- a/reports/2026-09-05.xlsx
+++ b/reports/2026-09-05.xlsx
@@ -767,13 +767,13 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" t="n">
         <v>3</v>
       </c>
-      <c r="C15" t="n">
-        <v>1</v>
-      </c>
       <c r="D15" t="n">
-        <v>-47.95</v>
+        <v>10.67</v>
       </c>
       <c r="E15" t="n">
         <v>-2.94</v>
@@ -812,13 +812,13 @@
         </is>
       </c>
       <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
         <v>2</v>
       </c>
-      <c r="C18" t="n">
-        <v>1</v>
-      </c>
       <c r="D18" t="n">
-        <v>-1.43</v>
+        <v>33.37</v>
       </c>
       <c r="E18" t="n">
         <v>19.6</v>
@@ -831,13 +831,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>-50.04</v>
+        <v>-26.22</v>
       </c>
       <c r="E19" t="n">
         <v>-2.94</v>
@@ -857,13 +857,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>-77.09</v>
+        <v>-42.29</v>
       </c>
       <c r="E21" t="n">
         <v>16.66</v>
@@ -876,13 +876,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>25.62</v>
+        <v>49.44</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -902,13 +902,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>-11.09</v>
+        <v>47.53</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>

</xml_diff>